<commit_message>
Host on chaitra6 Vercel project; tests target the new domain
- README: new live URLs and Git-based deploy flow
- E2E suite defaults to restaurant-table-booking-coral.vercel.app and waits
  for the booking form to initialise before picking a date
- Refreshed test report, screenshots and recording (30/30 passed)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test_Report.xlsx
+++ b/Test_Report.xlsx
@@ -20,13 +20,13 @@
     <t>Run date</t>
   </si>
   <si>
-    <t>22 Oct 2026, 13:49</t>
+    <t>22 Oct 2026, 17:31</t>
   </si>
   <si>
     <t>Target URL</t>
   </si>
   <si>
-    <t>https://restaurant-table-booking-omega.vercel.app</t>
+    <t>https://restaurant-table-booking-coral.vercel.app</t>
   </si>
   <si>
     <t>Backend</t>
@@ -62,7 +62,7 @@
     <t>Total duration</t>
   </si>
   <si>
-    <t>57.3 s</t>
+    <t>95.3 s</t>
   </si>
   <si>
     <t>Screenshots</t>
@@ -74,7 +74,7 @@
     <t>Screen recording</t>
   </si>
   <si>
-    <t>testing_recording/E2E_Test_Run_20261022_0819.mp4</t>
+    <t>testing_recording/E2E_Test_Run_20261022_1201.mp4</t>
   </si>
   <si>
     <t>ID</t>
@@ -1514,7 +1514,7 @@
         <v>40</v>
       </c>
       <c r="J2" s="4">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>41</v>
@@ -1549,7 +1549,7 @@
         <v>40</v>
       </c>
       <c r="J3" s="4">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>50</v>
@@ -1584,7 +1584,7 @@
         <v>40</v>
       </c>
       <c r="J4" s="4">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="K4" s="4" t="s">
         <v>58</v>
@@ -1619,7 +1619,7 @@
         <v>40</v>
       </c>
       <c r="J5" s="4">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>67</v>
@@ -1654,7 +1654,7 @@
         <v>40</v>
       </c>
       <c r="J6" s="4">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="K6" s="4" t="s">
         <v>75</v>
@@ -1689,7 +1689,7 @@
         <v>40</v>
       </c>
       <c r="J7" s="4">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>82</v>
@@ -1724,7 +1724,7 @@
         <v>40</v>
       </c>
       <c r="J8" s="4">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>89</v>
@@ -1759,7 +1759,7 @@
         <v>40</v>
       </c>
       <c r="J9" s="4">
-        <v>1</v>
+        <v>14.2</v>
       </c>
       <c r="K9" s="4" t="s">
         <v>97</v>
@@ -1794,7 +1794,7 @@
         <v>40</v>
       </c>
       <c r="J10" s="4">
-        <v>3</v>
+        <v>9.3</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>104</v>
@@ -1829,7 +1829,7 @@
         <v>40</v>
       </c>
       <c r="J11" s="4">
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="K11" s="4" t="s">
         <v>112</v>
@@ -1864,7 +1864,7 @@
         <v>40</v>
       </c>
       <c r="J12" s="4">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="K12" s="4" t="s">
         <v>118</v>
@@ -1899,7 +1899,7 @@
         <v>40</v>
       </c>
       <c r="J13" s="4">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="K13" s="4" t="s">
         <v>125</v>
@@ -1934,7 +1934,7 @@
         <v>40</v>
       </c>
       <c r="J14" s="4">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="K14" s="4" t="s">
         <v>133</v>
@@ -1969,7 +1969,7 @@
         <v>40</v>
       </c>
       <c r="J15" s="4">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="K15" s="4" t="s">
         <v>141</v>
@@ -2004,7 +2004,7 @@
         <v>40</v>
       </c>
       <c r="J16" s="4">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="K16" s="4" t="s">
         <v>149</v>
@@ -2039,7 +2039,7 @@
         <v>40</v>
       </c>
       <c r="J17" s="4">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="K17" s="4" t="s">
         <v>156</v>
@@ -2074,7 +2074,7 @@
         <v>40</v>
       </c>
       <c r="J18" s="4">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="K18" s="4" t="s">
         <v>163</v>
@@ -2109,7 +2109,7 @@
         <v>40</v>
       </c>
       <c r="J19" s="4">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="K19" s="4" t="s">
         <v>171</v>
@@ -2144,7 +2144,7 @@
         <v>40</v>
       </c>
       <c r="J20" s="4">
-        <v>1.6</v>
+        <v>2.5</v>
       </c>
       <c r="K20" s="4" t="s">
         <v>178</v>
@@ -2179,7 +2179,7 @@
         <v>40</v>
       </c>
       <c r="J21" s="4">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="K21" s="4" t="s">
         <v>185</v>
@@ -2214,7 +2214,7 @@
         <v>40</v>
       </c>
       <c r="J22" s="4">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="K22" s="4" t="s">
         <v>192</v>
@@ -2249,7 +2249,7 @@
         <v>40</v>
       </c>
       <c r="J23" s="4">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="K23" s="4" t="s">
         <v>200</v>
@@ -2284,7 +2284,7 @@
         <v>40</v>
       </c>
       <c r="J24" s="4">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="K24" s="4" t="s">
         <v>207</v>
@@ -2319,7 +2319,7 @@
         <v>40</v>
       </c>
       <c r="J25" s="4">
-        <v>2.1</v>
+        <v>2.9</v>
       </c>
       <c r="K25" s="4" t="s">
         <v>214</v>
@@ -2354,7 +2354,7 @@
         <v>40</v>
       </c>
       <c r="J26" s="4">
-        <v>3.4</v>
+        <v>5.3</v>
       </c>
       <c r="K26" s="4" t="s">
         <v>221</v>
@@ -2389,7 +2389,7 @@
         <v>40</v>
       </c>
       <c r="J27" s="4">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="K27" s="4" t="s">
         <v>227</v>
@@ -2424,7 +2424,7 @@
         <v>40</v>
       </c>
       <c r="J28" s="4">
-        <v>3.3</v>
+        <v>3.9</v>
       </c>
       <c r="K28" s="4" t="s">
         <v>234</v>
@@ -2494,7 +2494,7 @@
         <v>40</v>
       </c>
       <c r="J30" s="4">
-        <v>1.9</v>
+        <v>2.4</v>
       </c>
       <c r="K30" s="4" t="s">
         <v>248</v>
@@ -2529,7 +2529,7 @@
         <v>40</v>
       </c>
       <c r="J31" s="4">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
       <c r="K31" s="4" t="s">
         <v>255</v>

</xml_diff>